<commit_message>
Dodao sam svasta, generalno za master, tezu, dokumentaciju...
</commit_message>
<xml_diff>
--- a/project/results/experiment_results.xlsx
+++ b/project/results/experiment_results.xlsx
@@ -623,115 +623,115 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>set_1</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>N3C3W2_F.txt</t>
+          <t>Falkenauer_t60_17.txt</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="G2" t="n">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0008897781372070312</v>
+        <v>8.106231689453125e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0008161067962646484</v>
+        <v>8.988380432128906e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0005364418029785156</v>
+        <v>9.465217590332031e-05</v>
       </c>
       <c r="M2" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0008780956268310547</v>
+        <v>8.630752563476562e-05</v>
       </c>
       <c r="O2" t="n">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="P2" t="n">
-        <v>0.001346349716186523</v>
+        <v>0.0001001358032226562</v>
       </c>
       <c r="Q2" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="R2" t="n">
-        <v>0.001679182052612305</v>
+        <v>0.0001204013824462891</v>
       </c>
       <c r="S2" t="n">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0004866123199462891</v>
+        <v>0.0001091957092285156</v>
       </c>
       <c r="U2" t="n">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="V2" t="n">
-        <v>6.318092346191406e-05</v>
+        <v>1.955032348632812e-05</v>
       </c>
       <c r="W2" t="n">
-        <v>114</v>
+        <v>24</v>
       </c>
       <c r="X2" t="n">
-        <v>8.559226989746094e-05</v>
+        <v>2.6702880859375e-05</v>
       </c>
       <c r="Y2" t="n">
-        <v>114</v>
+        <v>24</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0001595020294189453</v>
+        <v>2.765655517578125e-05</v>
       </c>
       <c r="AA2" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.001399993896484375</v>
+        <v>9.179115295410156e-05</v>
       </c>
       <c r="AC2" t="n">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.001412868499755859</v>
+        <v>0.0001146793365478516</v>
       </c>
       <c r="AE2" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.00018310546875</v>
+        <v>7.128715515136719e-05</v>
       </c>
       <c r="AG2" t="n">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.0002911090850830078</v>
+        <v>5.269050598144531e-05</v>
       </c>
       <c r="AI2" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="AJ2" t="n">
-        <v>2.171562433242798</v>
+        <v>0.2078464031219482</v>
       </c>
       <c r="AK2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -742,115 +742,115 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>set_1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Falkenauer_u120_11.txt</t>
+          <t>N4C2W2_O.txt</t>
         </is>
       </c>
       <c r="D3" t="n">
+        <v>500</v>
+      </c>
+      <c r="E3" t="n">
         <v>120</v>
       </c>
-      <c r="E3" t="n">
-        <v>150</v>
-      </c>
       <c r="F3" t="n">
-        <v>49</v>
+        <v>253</v>
       </c>
       <c r="G3" t="n">
-        <v>52</v>
+        <v>253</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0003690719604492188</v>
+        <v>0.006803274154663086</v>
       </c>
       <c r="I3" t="n">
-        <v>50</v>
+        <v>253</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0003981590270996094</v>
+        <v>0.006093025207519531</v>
       </c>
       <c r="K3" t="n">
-        <v>52</v>
+        <v>253</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0003118515014648438</v>
+        <v>0.001612663269042969</v>
       </c>
       <c r="M3" t="n">
-        <v>50</v>
+        <v>253</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0003602504730224609</v>
+        <v>0.006740808486938477</v>
       </c>
       <c r="O3" t="n">
-        <v>51</v>
+        <v>253</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0005309581756591797</v>
+        <v>0.01076698303222656</v>
       </c>
       <c r="Q3" t="n">
-        <v>50</v>
+        <v>253</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0005383491516113281</v>
+        <v>0.01043248176574707</v>
       </c>
       <c r="S3" t="n">
-        <v>51</v>
+        <v>253</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0002586841583251953</v>
+        <v>0.0009565353393554688</v>
       </c>
       <c r="U3" t="n">
-        <v>63</v>
+        <v>344</v>
       </c>
       <c r="V3" t="n">
-        <v>3.600120544433594e-05</v>
+        <v>0.0002295970916748047</v>
       </c>
       <c r="W3" t="n">
-        <v>71</v>
+        <v>344</v>
       </c>
       <c r="X3" t="n">
-        <v>5.221366882324219e-05</v>
+        <v>0.0003032684326171875</v>
       </c>
       <c r="Y3" t="n">
-        <v>71</v>
+        <v>344</v>
       </c>
       <c r="Z3" t="n">
-        <v>9.72747802734375e-05</v>
+        <v>0.0004215240478515625</v>
       </c>
       <c r="AA3" t="n">
-        <v>56</v>
+        <v>253</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.000431060791015625</v>
+        <v>0.01087856292724609</v>
       </c>
       <c r="AC3" t="n">
-        <v>51</v>
+        <v>253</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.0005459785461425781</v>
+        <v>0.01082301139831543</v>
       </c>
       <c r="AE3" t="n">
-        <v>56</v>
+        <v>253</v>
       </c>
       <c r="AF3" t="n">
-        <v>9.965896606445312e-05</v>
+        <v>0.0004603862762451172</v>
       </c>
       <c r="AG3" t="n">
-        <v>51</v>
+        <v>253</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.0001060962677001953</v>
+        <v>0.0004723072052001953</v>
       </c>
       <c r="AI3" t="n">
-        <v>50</v>
+        <v>253</v>
       </c>
       <c r="AJ3" t="n">
-        <v>1.276925802230835</v>
+        <v>13.60601019859314</v>
       </c>
       <c r="AK3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -861,115 +861,115 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>set_1</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>N4C2W4_H.txt</t>
+          <t>Falkenauer_t60_03.txt</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="E4" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="H4" t="n">
-        <v>0.008208990097045898</v>
+        <v>9.870529174804688e-05</v>
       </c>
       <c r="I4" t="n">
-        <v>296</v>
+        <v>23</v>
       </c>
       <c r="J4" t="n">
-        <v>0.008051395416259766</v>
+        <v>8.559226989746094e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="L4" t="n">
-        <v>0.002274990081787109</v>
+        <v>9.202957153320312e-05</v>
       </c>
       <c r="M4" t="n">
-        <v>296</v>
+        <v>23</v>
       </c>
       <c r="N4" t="n">
-        <v>0.008258819580078125</v>
+        <v>8.249282836914062e-05</v>
       </c>
       <c r="O4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="P4" t="n">
-        <v>0.01153278350830078</v>
+        <v>0.0001122951507568359</v>
       </c>
       <c r="Q4" t="n">
-        <v>296</v>
+        <v>23</v>
       </c>
       <c r="R4" t="n">
-        <v>0.01363229751586914</v>
+        <v>0.0001223087310791016</v>
       </c>
       <c r="S4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="T4" t="n">
-        <v>0.001118183135986328</v>
+        <v>0.0001101493835449219</v>
       </c>
       <c r="U4" t="n">
-        <v>385</v>
+        <v>20</v>
       </c>
       <c r="V4" t="n">
-        <v>0.0002105236053466797</v>
+        <v>1.835823059082031e-05</v>
       </c>
       <c r="W4" t="n">
-        <v>385</v>
+        <v>25</v>
       </c>
       <c r="X4" t="n">
-        <v>0.0002756118774414062</v>
+        <v>2.694129943847656e-05</v>
       </c>
       <c r="Y4" t="n">
-        <v>385</v>
+        <v>25</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.0005249977111816406</v>
+        <v>2.717971801757812e-05</v>
       </c>
       <c r="AA4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.01167416572570801</v>
+        <v>0.0001277923583984375</v>
       </c>
       <c r="AC4" t="n">
-        <v>296</v>
+        <v>23</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.01408076286315918</v>
+        <v>0.0001149177551269531</v>
       </c>
       <c r="AE4" t="n">
-        <v>296</v>
+        <v>20</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.0005102157592773438</v>
+        <v>4.839897155761719e-05</v>
       </c>
       <c r="AG4" t="n">
-        <v>296</v>
+        <v>23</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.0005903244018554688</v>
+        <v>5.221366882324219e-05</v>
       </c>
       <c r="AI4" t="n">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="AJ4" t="n">
-        <v>15.78590869903564</v>
+        <v>0.2137737274169922</v>
       </c>
       <c r="AK4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -980,115 +980,115 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>set_1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Falkenauer_u120_05.txt</t>
+          <t>N4C1W4_Q.txt</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>120</v>
+        <v>500</v>
       </c>
       <c r="E5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>48</v>
+        <v>359</v>
       </c>
       <c r="G5" t="n">
-        <v>52</v>
+        <v>359</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0003054141998291016</v>
+        <v>0.008267641067504883</v>
       </c>
       <c r="I5" t="n">
-        <v>49</v>
+        <v>359</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0003190040588378906</v>
+        <v>0.009367942810058594</v>
       </c>
       <c r="K5" t="n">
-        <v>52</v>
+        <v>359</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0002455711364746094</v>
+        <v>0.001767158508300781</v>
       </c>
       <c r="M5" t="n">
-        <v>49</v>
+        <v>359</v>
       </c>
       <c r="N5" t="n">
-        <v>0.0003495216369628906</v>
+        <v>0.009973049163818359</v>
       </c>
       <c r="O5" t="n">
-        <v>52</v>
+        <v>359</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0003993511199951172</v>
+        <v>0.01574134826660156</v>
       </c>
       <c r="Q5" t="n">
-        <v>49</v>
+        <v>359</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0005948543548583984</v>
+        <v>0.01447010040283203</v>
       </c>
       <c r="S5" t="n">
-        <v>52</v>
+        <v>359</v>
       </c>
       <c r="T5" t="n">
-        <v>0.0002827644348144531</v>
+        <v>0.0007085800170898438</v>
       </c>
       <c r="U5" t="n">
-        <v>61</v>
+        <v>423</v>
       </c>
       <c r="V5" t="n">
-        <v>3.671646118164062e-05</v>
+        <v>0.0002007484436035156</v>
       </c>
       <c r="W5" t="n">
-        <v>68</v>
+        <v>423</v>
       </c>
       <c r="X5" t="n">
-        <v>6.055831909179688e-05</v>
+        <v>0.0002577304840087891</v>
       </c>
       <c r="Y5" t="n">
-        <v>68</v>
+        <v>423</v>
       </c>
       <c r="Z5" t="n">
-        <v>9.775161743164062e-05</v>
+        <v>0.0008146762847900391</v>
       </c>
       <c r="AA5" t="n">
-        <v>54</v>
+        <v>359</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.0003952980041503906</v>
+        <v>0.01445174217224121</v>
       </c>
       <c r="AC5" t="n">
-        <v>50</v>
+        <v>359</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.0005474090576171875</v>
+        <v>0.01314091682434082</v>
       </c>
       <c r="AE5" t="n">
-        <v>54</v>
+        <v>359</v>
       </c>
       <c r="AF5" t="n">
-        <v>9.298324584960938e-05</v>
+        <v>0.0006265640258789062</v>
       </c>
       <c r="AG5" t="n">
-        <v>50</v>
+        <v>359</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.0001044273376464844</v>
+        <v>0.0004456043243408203</v>
       </c>
       <c r="AI5" t="n">
-        <v>49</v>
+        <v>359</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.8474185466766357</v>
+        <v>21.61660766601562</v>
       </c>
       <c r="AK5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1099,115 +1099,115 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>set_1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Falkenauer_t501_06.txt</t>
+          <t>N4C3W2_B.txt</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F6" t="n">
-        <v>167</v>
+        <v>203</v>
       </c>
       <c r="G6" t="n">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00344538688659668</v>
+        <v>0.004851818084716797</v>
       </c>
       <c r="I6" t="n">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="J6" t="n">
-        <v>0.004434823989868164</v>
+        <v>0.004589080810546875</v>
       </c>
       <c r="K6" t="n">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="L6" t="n">
-        <v>0.002250194549560547</v>
+        <v>0.001220703125</v>
       </c>
       <c r="M6" t="n">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="N6" t="n">
-        <v>0.004268407821655273</v>
+        <v>0.004875898361206055</v>
       </c>
       <c r="O6" t="n">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="P6" t="n">
-        <v>0.004708290100097656</v>
+        <v>0.008093595504760742</v>
       </c>
       <c r="Q6" t="n">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="R6" t="n">
-        <v>0.006044149398803711</v>
+        <v>0.008060455322265625</v>
       </c>
       <c r="S6" t="n">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="T6" t="n">
-        <v>0.0009136199951171875</v>
+        <v>0.001007795333862305</v>
       </c>
       <c r="U6" t="n">
-        <v>167</v>
+        <v>288</v>
       </c>
       <c r="V6" t="n">
-        <v>0.0001494884490966797</v>
+        <v>0.0001587867736816406</v>
       </c>
       <c r="W6" t="n">
-        <v>202</v>
+        <v>288</v>
       </c>
       <c r="X6" t="n">
-        <v>0.0002498626708984375</v>
+        <v>0.0002079010009765625</v>
       </c>
       <c r="Y6" t="n">
-        <v>202</v>
+        <v>288</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.0002815723419189453</v>
+        <v>0.0003974437713623047</v>
       </c>
       <c r="AA6" t="n">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.004584789276123047</v>
+        <v>0.008050441741943359</v>
       </c>
       <c r="AC6" t="n">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.006082773208618164</v>
+        <v>0.008051633834838867</v>
       </c>
       <c r="AE6" t="n">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.0005581378936767578</v>
+        <v>0.0004796981811523438</v>
       </c>
       <c r="AG6" t="n">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.0005729198455810547</v>
+        <v>0.0004851818084716797</v>
       </c>
       <c r="AI6" t="n">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="AJ6" t="n">
-        <v>10.48444414138794</v>
+        <v>13.10856533050537</v>
       </c>
       <c r="AK6" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1223,107 +1223,107 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>N2C2W4_B.txt</t>
+          <t>N3C2W4_P.txt</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E7" t="n">
         <v>120</v>
       </c>
       <c r="F7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="G7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0004403591156005859</v>
+        <v>0.00113368034362793</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="J7" t="n">
-        <v>0.000354766845703125</v>
+        <v>0.001149415969848633</v>
       </c>
       <c r="K7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0002744197845458984</v>
+        <v>0.0005600452423095703</v>
       </c>
       <c r="M7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0003561973571777344</v>
+        <v>0.001237869262695312</v>
       </c>
       <c r="O7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0005590915679931641</v>
+        <v>0.00184178352355957</v>
       </c>
       <c r="Q7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0005059242248535156</v>
+        <v>0.001852989196777344</v>
       </c>
       <c r="S7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="T7" t="n">
-        <v>0.0001943111419677734</v>
+        <v>0.0003492832183837891</v>
       </c>
       <c r="U7" t="n">
-        <v>75</v>
+        <v>151</v>
       </c>
       <c r="V7" t="n">
-        <v>3.170967102050781e-05</v>
+        <v>9.369850158691406e-05</v>
       </c>
       <c r="W7" t="n">
-        <v>75</v>
+        <v>151</v>
       </c>
       <c r="X7" t="n">
-        <v>4.124641418457031e-05</v>
+        <v>0.0001056194305419922</v>
       </c>
       <c r="Y7" t="n">
-        <v>75</v>
+        <v>151</v>
       </c>
       <c r="Z7" t="n">
-        <v>8.654594421386719e-05</v>
+        <v>0.0001642704010009766</v>
       </c>
       <c r="AA7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.0004982948303222656</v>
+        <v>0.001905202865600586</v>
       </c>
       <c r="AC7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.000652313232421875</v>
+        <v>0.001879453659057617</v>
       </c>
       <c r="AE7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.0001091957092285156</v>
+        <v>0.0001599788665771484</v>
       </c>
       <c r="AG7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.0001089572906494141</v>
+        <v>0.0001745223999023438</v>
       </c>
       <c r="AI7" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="AJ7" t="n">
-        <v>1.269204139709473</v>
+        <v>3.475831985473633</v>
       </c>
       <c r="AK7" t="n">
         <v>0</v>
@@ -1337,115 +1337,115 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>set_1</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N4C3W4_G.txt</t>
+          <t>Falkenauer_t120_02.txt</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>500</v>
+        <v>120</v>
       </c>
       <c r="E8" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>222</v>
+        <v>40</v>
       </c>
       <c r="G8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="H8" t="n">
-        <v>0.005005598068237305</v>
+        <v>0.0002541542053222656</v>
       </c>
       <c r="I8" t="n">
-        <v>226</v>
+        <v>45</v>
       </c>
       <c r="J8" t="n">
-        <v>0.004814386367797852</v>
+        <v>0.0004379749298095703</v>
       </c>
       <c r="K8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>0.001313924789428711</v>
+        <v>0.0003347396850585938</v>
       </c>
       <c r="M8" t="n">
-        <v>226</v>
+        <v>45</v>
       </c>
       <c r="N8" t="n">
-        <v>0.006113767623901367</v>
+        <v>0.0002765655517578125</v>
       </c>
       <c r="O8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="P8" t="n">
-        <v>0.008535385131835938</v>
+        <v>0.00032806396484375</v>
       </c>
       <c r="Q8" t="n">
-        <v>226</v>
+        <v>45</v>
       </c>
       <c r="R8" t="n">
-        <v>0.008712530136108398</v>
+        <v>0.0004038810729980469</v>
       </c>
       <c r="S8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="T8" t="n">
-        <v>0.001275062561035156</v>
+        <v>0.0002157688140869141</v>
       </c>
       <c r="U8" t="n">
-        <v>313</v>
+        <v>40</v>
       </c>
       <c r="V8" t="n">
-        <v>0.0001990795135498047</v>
+        <v>3.457069396972656e-05</v>
       </c>
       <c r="W8" t="n">
-        <v>313</v>
+        <v>49</v>
       </c>
       <c r="X8" t="n">
-        <v>0.0002648830413818359</v>
+        <v>5.245208740234375e-05</v>
       </c>
       <c r="Y8" t="n">
-        <v>313</v>
+        <v>49</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.0004777908325195312</v>
+        <v>5.173683166503906e-05</v>
       </c>
       <c r="AA8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.01057767868041992</v>
+        <v>0.0003530979156494141</v>
       </c>
       <c r="AC8" t="n">
-        <v>226</v>
+        <v>45</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.0109717845916748</v>
+        <v>0.0006341934204101562</v>
       </c>
       <c r="AE8" t="n">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.0004868507385253906</v>
+        <v>0.0001068115234375</v>
       </c>
       <c r="AG8" t="n">
-        <v>226</v>
+        <v>45</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.0005967617034912109</v>
+        <v>0.0002584457397460938</v>
       </c>
       <c r="AI8" t="n">
-        <v>234</v>
+        <v>40</v>
       </c>
       <c r="AJ8" t="n">
-        <v>13.15340733528137</v>
+        <v>0.7091286182403564</v>
       </c>
       <c r="AK8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1456,115 +1456,115 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Falkenauer_u250_10.txt</t>
+          <t>Falkenauer_t249_09.txt</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E9" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="G9" t="n">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="H9" t="n">
-        <v>0.001317977905273438</v>
+        <v>0.0008924007415771484</v>
       </c>
       <c r="I9" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001334190368652344</v>
+        <v>0.001055479049682617</v>
       </c>
       <c r="K9" t="n">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0007138252258300781</v>
+        <v>0.0007791519165039062</v>
       </c>
       <c r="M9" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N9" t="n">
-        <v>0.00139617919921875</v>
+        <v>0.001058816909790039</v>
       </c>
       <c r="O9" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="P9" t="n">
-        <v>0.001580476760864258</v>
+        <v>0.001172542572021484</v>
       </c>
       <c r="Q9" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="R9" t="n">
-        <v>0.00217127799987793</v>
+        <v>0.00148773193359375</v>
       </c>
       <c r="S9" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="T9" t="n">
-        <v>0.0005280971527099609</v>
+        <v>0.0004012584686279297</v>
       </c>
       <c r="U9" t="n">
-        <v>137</v>
+        <v>83</v>
       </c>
       <c r="V9" t="n">
-        <v>7.748603820800781e-05</v>
+        <v>7.176399230957031e-05</v>
       </c>
       <c r="W9" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="X9" t="n">
-        <v>0.0001206398010253906</v>
+        <v>0.0001099109649658203</v>
       </c>
       <c r="Y9" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.0002048015594482422</v>
+        <v>0.0001089572906494141</v>
       </c>
       <c r="AA9" t="n">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.001774072647094727</v>
+        <v>0.001116514205932617</v>
       </c>
       <c r="AC9" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.002200841903686523</v>
+        <v>0.001500606536865234</v>
       </c>
       <c r="AE9" t="n">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.0002117156982421875</v>
+        <v>0.0002510547637939453</v>
       </c>
       <c r="AG9" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.0002398490905761719</v>
+        <v>0.0002543926239013672</v>
       </c>
       <c r="AI9" t="n">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="AJ9" t="n">
-        <v>3.677238941192627</v>
+        <v>2.712917327880859</v>
       </c>
       <c r="AK9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1575,115 +1575,115 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>set_1</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N2C1W4_T.txt</t>
+          <t>Falkenauer_t60_14.txt</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="G10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0004031658172607422</v>
+        <v>7.867813110351562e-05</v>
       </c>
       <c r="I10" t="n">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0003659725189208984</v>
+        <v>8.797645568847656e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0002489089965820312</v>
+        <v>9.584426879882812e-05</v>
       </c>
       <c r="M10" t="n">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0004107952117919922</v>
+        <v>8.606910705566406e-05</v>
       </c>
       <c r="O10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="P10" t="n">
-        <v>0.0005936622619628906</v>
+        <v>0.0001013278961181641</v>
       </c>
       <c r="Q10" t="n">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="R10" t="n">
-        <v>0.0005190372467041016</v>
+        <v>0.0002717971801757812</v>
       </c>
       <c r="S10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0001478195190429688</v>
+        <v>0.0001184940338134766</v>
       </c>
       <c r="U10" t="n">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="V10" t="n">
-        <v>3.0517578125e-05</v>
+        <v>1.835823059082031e-05</v>
       </c>
       <c r="W10" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
       <c r="X10" t="n">
-        <v>3.910064697265625e-05</v>
+        <v>2.813339233398438e-05</v>
       </c>
       <c r="Y10" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
       <c r="Z10" t="n">
-        <v>8.535385131835938e-05</v>
+        <v>2.741813659667969e-05</v>
       </c>
       <c r="AA10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.0005304813385009766</v>
+        <v>9.012222290039062e-05</v>
       </c>
       <c r="AC10" t="n">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.0005276203155517578</v>
+        <v>0.0001165866851806641</v>
       </c>
       <c r="AE10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="AF10" t="n">
-        <v>8.130073547363281e-05</v>
+        <v>0.0001113414764404297</v>
       </c>
       <c r="AG10" t="n">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="AH10" t="n">
-        <v>8.058547973632812e-05</v>
+        <v>5.197525024414062e-05</v>
       </c>
       <c r="AI10" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="AJ10" t="n">
-        <v>1.18154501914978</v>
+        <v>0.2106759548187256</v>
       </c>
       <c r="AK10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1699,110 +1699,110 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>N3C2W1_B.txt</t>
+          <t>N1C2W4_G.txt</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
         <v>120</v>
       </c>
       <c r="F11" t="n">
-        <v>82</v>
+        <v>30</v>
       </c>
       <c r="G11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001185178756713867</v>
+        <v>9.894371032714844e-05</v>
       </c>
       <c r="I11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0009295940399169922</v>
+        <v>8.797645568847656e-05</v>
       </c>
       <c r="K11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0005712509155273438</v>
+        <v>9.1552734375e-05</v>
       </c>
       <c r="M11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="N11" t="n">
-        <v>0.0008697509765625</v>
+        <v>0.0001235008239746094</v>
       </c>
       <c r="O11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="P11" t="n">
-        <v>0.001821756362915039</v>
+        <v>0.0001385211944580078</v>
       </c>
       <c r="Q11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="R11" t="n">
-        <v>0.001851081848144531</v>
+        <v>0.0001382827758789062</v>
       </c>
       <c r="S11" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0005161762237548828</v>
+        <v>0.0001018047332763672</v>
       </c>
       <c r="U11" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="V11" t="n">
-        <v>7.963180541992188e-05</v>
+        <v>1.621246337890625e-05</v>
       </c>
       <c r="W11" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="X11" t="n">
-        <v>9.274482727050781e-05</v>
+        <v>2.050399780273438e-05</v>
       </c>
       <c r="Y11" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.0001683235168457031</v>
+        <v>4.887580871582031e-05</v>
       </c>
       <c r="AA11" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.001565456390380859</v>
+        <v>0.0001282691955566406</v>
       </c>
       <c r="AC11" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.001758575439453125</v>
+        <v>0.0001327991485595703</v>
       </c>
       <c r="AE11" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.0002381801605224609</v>
+        <v>3.933906555175781e-05</v>
       </c>
       <c r="AG11" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.0002262592315673828</v>
+        <v>3.933906555175781e-05</v>
       </c>
       <c r="AI11" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="AJ11" t="n">
-        <v>2.32247519493103</v>
+        <v>0.4849312305450439</v>
       </c>
       <c r="AK11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1818,107 +1818,107 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>N3W3B2R7.txt</t>
+          <t>N1W3B3R9.txt</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="E12" t="n">
         <v>1000</v>
       </c>
       <c r="F12" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0005507469177246094</v>
+        <v>7.390975952148438e-05</v>
       </c>
       <c r="I12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0004088878631591797</v>
+        <v>0.0002832412719726562</v>
       </c>
       <c r="K12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0003302097320556641</v>
+        <v>7.295608520507812e-05</v>
       </c>
       <c r="M12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0004332065582275391</v>
+        <v>8.7738037109375e-05</v>
       </c>
       <c r="O12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="P12" t="n">
-        <v>0.0005185604095458984</v>
+        <v>7.677078247070312e-05</v>
       </c>
       <c r="Q12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="R12" t="n">
-        <v>0.0005970001220703125</v>
+        <v>6.461143493652344e-05</v>
       </c>
       <c r="S12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="T12" t="n">
-        <v>0.004913091659545898</v>
+        <v>0.0009810924530029297</v>
       </c>
       <c r="U12" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="V12" t="n">
-        <v>5.698204040527344e-05</v>
+        <v>1.502037048339844e-05</v>
       </c>
       <c r="W12" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="X12" t="n">
-        <v>7.987022399902344e-05</v>
+        <v>2.026557922363281e-05</v>
       </c>
       <c r="Y12" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.0002624988555908203</v>
+        <v>6.413459777832031e-05</v>
       </c>
       <c r="AA12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.0004506111145019531</v>
+        <v>5.125999450683594e-05</v>
       </c>
       <c r="AC12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.0005571842193603516</v>
+        <v>5.555152893066406e-05</v>
       </c>
       <c r="AE12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.0002298355102539062</v>
+        <v>3.719329833984375e-05</v>
       </c>
       <c r="AG12" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.0001692771911621094</v>
+        <v>3.838539123535156e-05</v>
       </c>
       <c r="AI12" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="AJ12" t="n">
-        <v>1.123782634735107</v>
+        <v>0.1187021732330322</v>
       </c>
       <c r="AK12" t="n">
         <v>0</v>
@@ -1937,107 +1937,107 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>N4W4B1R6.txt</t>
+          <t>N3W1B1R0.txt</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="E13" t="n">
         <v>1000</v>
       </c>
       <c r="F13" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="G13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="H13" t="n">
-        <v>0.001405954360961914</v>
+        <v>0.000701904296875</v>
       </c>
       <c r="I13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="J13" t="n">
-        <v>0.001455068588256836</v>
+        <v>0.0006890296936035156</v>
       </c>
       <c r="K13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0005574226379394531</v>
+        <v>0.0005278587341308594</v>
       </c>
       <c r="M13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="N13" t="n">
-        <v>0.001947164535522461</v>
+        <v>0.0008602142333984375</v>
       </c>
       <c r="O13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="P13" t="n">
-        <v>0.001930475234985352</v>
+        <v>0.001009225845336914</v>
       </c>
       <c r="Q13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="R13" t="n">
-        <v>0.0019378662109375</v>
+        <v>0.001018047332763672</v>
       </c>
       <c r="S13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="T13" t="n">
-        <v>0.01069307327270508</v>
+        <v>0.003891468048095703</v>
       </c>
       <c r="U13" t="n">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="V13" t="n">
-        <v>0.0001454353332519531</v>
+        <v>6.031990051269531e-05</v>
       </c>
       <c r="W13" t="n">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="X13" t="n">
-        <v>0.000263214111328125</v>
+        <v>8.273124694824219e-05</v>
       </c>
       <c r="Y13" t="n">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.0004565715789794922</v>
+        <v>0.0002193450927734375</v>
       </c>
       <c r="AA13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.002341032028198242</v>
+        <v>0.0009541511535644531</v>
       </c>
       <c r="AC13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.002408266067504883</v>
+        <v>0.001010656356811523</v>
       </c>
       <c r="AE13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.0005154609680175781</v>
+        <v>0.0001573562622070312</v>
       </c>
       <c r="AG13" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.000576019287109375</v>
+        <v>0.0001730918884277344</v>
       </c>
       <c r="AI13" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="AJ13" t="n">
-        <v>3.940504312515259</v>
+        <v>1.847396850585938</v>
       </c>
       <c r="AK13" t="n">
         <v>2</v>
@@ -2056,110 +2056,110 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>N1W2B1R3.txt</t>
+          <t>N4W2B2R8.txt</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E14" t="n">
         <v>1000</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="H14" t="n">
-        <v>7.677078247070312e-05</v>
+        <v>0.00229644775390625</v>
       </c>
       <c r="I14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="J14" t="n">
-        <v>5.006790161132812e-05</v>
+        <v>0.002378702163696289</v>
       </c>
       <c r="K14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="L14" t="n">
-        <v>6.127357482910156e-05</v>
+        <v>0.001283407211303711</v>
       </c>
       <c r="M14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0001027584075927734</v>
+        <v>0.002613544464111328</v>
       </c>
       <c r="O14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="P14" t="n">
-        <v>6.985664367675781e-05</v>
+        <v>0.0034942626953125</v>
       </c>
       <c r="Q14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="R14" t="n">
-        <v>7.05718994140625e-05</v>
+        <v>0.003535032272338867</v>
       </c>
       <c r="S14" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="T14" t="n">
-        <v>0.001526117324829102</v>
+        <v>0.01014900207519531</v>
       </c>
       <c r="U14" t="n">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="V14" t="n">
-        <v>1.645088195800781e-05</v>
+        <v>0.0001521110534667969</v>
       </c>
       <c r="W14" t="n">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="X14" t="n">
-        <v>2.193450927734375e-05</v>
+        <v>0.0002064704895019531</v>
       </c>
       <c r="Y14" t="n">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="Z14" t="n">
-        <v>6.413459777832031e-05</v>
+        <v>0.0003979206085205078</v>
       </c>
       <c r="AA14" t="n">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="AB14" t="n">
-        <v>5.865097045898438e-05</v>
+        <v>0.003627538681030273</v>
       </c>
       <c r="AC14" t="n">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="AD14" t="n">
-        <v>6.318092346191406e-05</v>
+        <v>0.003581762313842773</v>
       </c>
       <c r="AE14" t="n">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="AF14" t="n">
-        <v>4.124641418457031e-05</v>
+        <v>0.0004391670227050781</v>
       </c>
       <c r="AG14" t="n">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="AH14" t="n">
-        <v>4.100799560546875e-05</v>
+        <v>0.0004668235778808594</v>
       </c>
       <c r="AI14" t="n">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.1314933300018311</v>
+        <v>6.427027463912964</v>
       </c>
       <c r="AK14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>N4W2B2R5.txt</t>
+          <t>N4W3B2R1.txt</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -2185,100 +2185,100 @@
         <v>1000</v>
       </c>
       <c r="F15" t="n">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="G15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="H15" t="n">
-        <v>0.002523660659790039</v>
+        <v>0.001752138137817383</v>
       </c>
       <c r="I15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="J15" t="n">
-        <v>0.002387046813964844</v>
+        <v>0.002240657806396484</v>
       </c>
       <c r="K15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="L15" t="n">
-        <v>0.001326322555541992</v>
+        <v>0.001071453094482422</v>
       </c>
       <c r="M15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="N15" t="n">
-        <v>0.002639293670654297</v>
+        <v>0.0019683837890625</v>
       </c>
       <c r="O15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="P15" t="n">
-        <v>0.003974676132202148</v>
+        <v>0.00243687629699707</v>
       </c>
       <c r="Q15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="R15" t="n">
-        <v>0.004030704498291016</v>
+        <v>0.002536773681640625</v>
       </c>
       <c r="S15" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="T15" t="n">
-        <v>0.01680183410644531</v>
+        <v>0.01000261306762695</v>
       </c>
       <c r="U15" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="V15" t="n">
-        <v>0.0001645088195800781</v>
+        <v>0.0001397132873535156</v>
       </c>
       <c r="W15" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="X15" t="n">
-        <v>0.0002083778381347656</v>
+        <v>0.0001959800720214844</v>
       </c>
       <c r="Y15" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.0004186630249023438</v>
+        <v>0.0003769397735595703</v>
       </c>
       <c r="AA15" t="n">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.004454612731933594</v>
+        <v>0.002768993377685547</v>
       </c>
       <c r="AC15" t="n">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.004728555679321289</v>
+        <v>0.002530336380004883</v>
       </c>
       <c r="AE15" t="n">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.0006213188171386719</v>
+        <v>0.0004403591156005859</v>
       </c>
       <c r="AG15" t="n">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="AH15" t="n">
-        <v>0.0009124279022216797</v>
+        <v>0.0004801750183105469</v>
       </c>
       <c r="AI15" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="AJ15" t="n">
-        <v>6.57194185256958</v>
+        <v>4.529487371444702</v>
       </c>
       <c r="AK15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2294,110 +2294,110 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>N2W2B2R8.txt</t>
+          <t>N3W2B2R2.txt</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E16" t="n">
         <v>1000</v>
       </c>
       <c r="F16" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0001919269561767578</v>
+        <v>0.0004951953887939453</v>
       </c>
       <c r="I16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0002548694610595703</v>
+        <v>0.0004246234893798828</v>
       </c>
       <c r="K16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="L16" t="n">
-        <v>0.0002501010894775391</v>
+        <v>0.0003848075866699219</v>
       </c>
       <c r="M16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="N16" t="n">
-        <v>0.0002169609069824219</v>
+        <v>0.0005393028259277344</v>
       </c>
       <c r="O16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="P16" t="n">
-        <v>0.0003037452697753906</v>
+        <v>0.0006275177001953125</v>
       </c>
       <c r="Q16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0003099441528320312</v>
+        <v>0.0006668567657470703</v>
       </c>
       <c r="S16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="T16" t="n">
-        <v>0.002165555953979492</v>
+        <v>0.004974365234375</v>
       </c>
       <c r="U16" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="V16" t="n">
-        <v>3.027915954589844e-05</v>
+        <v>6.389617919921875e-05</v>
       </c>
       <c r="W16" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="X16" t="n">
-        <v>4.315376281738281e-05</v>
+        <v>8.678436279296875e-05</v>
       </c>
       <c r="Y16" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.0001084804534912109</v>
+        <v>0.0001785755157470703</v>
       </c>
       <c r="AA16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.0001859664916992188</v>
+        <v>0.0006134510040283203</v>
       </c>
       <c r="AC16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.0002033710479736328</v>
+        <v>0.0006284713745117188</v>
       </c>
       <c r="AE16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="AF16" t="n">
-        <v>7.82012939453125e-05</v>
+        <v>0.0001623630523681641</v>
       </c>
       <c r="AG16" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="AH16" t="n">
-        <v>8.463859558105469e-05</v>
+        <v>0.0001707077026367188</v>
       </c>
       <c r="AI16" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.6897997856140137</v>
+        <v>1.31282901763916</v>
       </c>
       <c r="AK16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>N2W4B1R7.txt</t>
+          <t>N2W2B3R4.txt</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -2423,97 +2423,97 @@
         <v>1000</v>
       </c>
       <c r="F17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="G17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0001456737518310547</v>
+        <v>0.000164031982421875</v>
       </c>
       <c r="I17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="J17" t="n">
-        <v>9.918212890625e-05</v>
+        <v>0.0001461505889892578</v>
       </c>
       <c r="K17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="L17" t="n">
-        <v>9.846687316894531e-05</v>
+        <v>0.0001761913299560547</v>
       </c>
       <c r="M17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0001516342163085938</v>
+        <v>0.0002331733703613281</v>
       </c>
       <c r="O17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="P17" t="n">
-        <v>0.000133514404296875</v>
+        <v>0.0002155303955078125</v>
       </c>
       <c r="Q17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="R17" t="n">
-        <v>0.0001442432403564453</v>
+        <v>0.0002329349517822266</v>
       </c>
       <c r="S17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="T17" t="n">
-        <v>0.002391338348388672</v>
+        <v>0.002088546752929688</v>
       </c>
       <c r="U17" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="V17" t="n">
-        <v>3.194808959960938e-05</v>
+        <v>3.218650817871094e-05</v>
       </c>
       <c r="W17" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="X17" t="n">
-        <v>4.38690185546875e-05</v>
+        <v>4.410743713378906e-05</v>
       </c>
       <c r="Y17" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="Z17" t="n">
-        <v>8.654594421386719e-05</v>
+        <v>0.0001213550567626953</v>
       </c>
       <c r="AA17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.0001263618469238281</v>
+        <v>0.0002048015594482422</v>
       </c>
       <c r="AC17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.0001263618469238281</v>
+        <v>0.0002110004425048828</v>
       </c>
       <c r="AE17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AF17" t="n">
-        <v>7.295608520507812e-05</v>
+        <v>7.891654968261719e-05</v>
       </c>
       <c r="AG17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AH17" t="n">
-        <v>9.703636169433594e-05</v>
+        <v>8.440017700195312e-05</v>
       </c>
       <c r="AI17" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.2655935287475586</v>
+        <v>0.4058706760406494</v>
       </c>
       <c r="AK17" t="n">
         <v>0</v>
@@ -2532,110 +2532,110 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>N1W1B3R6.txt</t>
+          <t>N2W1B3R1.txt</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E18" t="n">
         <v>1000</v>
       </c>
       <c r="F18" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H18" t="n">
-        <v>7.486343383789062e-05</v>
+        <v>0.0002181529998779297</v>
       </c>
       <c r="I18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="J18" t="n">
-        <v>6.508827209472656e-05</v>
+        <v>0.0002076625823974609</v>
       </c>
       <c r="K18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="L18" t="n">
-        <v>8.511543273925781e-05</v>
+        <v>0.0002460479736328125</v>
       </c>
       <c r="M18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="N18" t="n">
-        <v>0.0002574920654296875</v>
+        <v>0.0003602504730224609</v>
       </c>
       <c r="O18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="P18" t="n">
-        <v>9.870529174804688e-05</v>
+        <v>0.0003235340118408203</v>
       </c>
       <c r="Q18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="R18" t="n">
-        <v>9.894371032714844e-05</v>
+        <v>0.0003199577331542969</v>
       </c>
       <c r="S18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="T18" t="n">
-        <v>0.001622676849365234</v>
+        <v>0.002004861831665039</v>
       </c>
       <c r="U18" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="V18" t="n">
-        <v>2.956390380859375e-05</v>
+        <v>3.170967102050781e-05</v>
       </c>
       <c r="W18" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="X18" t="n">
-        <v>3.838539123535156e-05</v>
+        <v>4.506111145019531e-05</v>
       </c>
       <c r="Y18" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.0001773834228515625</v>
+        <v>0.0001919269561767578</v>
       </c>
       <c r="AA18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.0001299381256103516</v>
+        <v>0.0002987384796142578</v>
       </c>
       <c r="AC18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AD18" t="n">
-        <v>0.0001461505889892578</v>
+        <v>0.0003237724304199219</v>
       </c>
       <c r="AE18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AF18" t="n">
-        <v>6.389617919921875e-05</v>
+        <v>8.153915405273438e-05</v>
       </c>
       <c r="AG18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AH18" t="n">
-        <v>6.079673767089844e-05</v>
+        <v>8.726119995117188e-05</v>
       </c>
       <c r="AI18" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.1641335487365723</v>
+        <v>0.6509764194488525</v>
       </c>
       <c r="AK18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2651,107 +2651,107 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>N4W4B3R7.txt</t>
+          <t>N1W1B3R5.txt</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="E19" t="n">
         <v>1000</v>
       </c>
       <c r="F19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="G19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="H19" t="n">
-        <v>0.001695394515991211</v>
+        <v>7.033348083496094e-05</v>
       </c>
       <c r="I19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="J19" t="n">
-        <v>0.001586198806762695</v>
+        <v>7.796287536621094e-05</v>
       </c>
       <c r="K19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0009965896606445312</v>
+        <v>0.0001094341278076172</v>
       </c>
       <c r="M19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="N19" t="n">
-        <v>0.001755714416503906</v>
+        <v>0.0001709461212158203</v>
       </c>
       <c r="O19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="P19" t="n">
-        <v>0.002267837524414062</v>
+        <v>9.751319885253906e-05</v>
       </c>
       <c r="Q19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="R19" t="n">
-        <v>0.002307653427124023</v>
+        <v>9.775161743164062e-05</v>
       </c>
       <c r="S19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="T19" t="n">
-        <v>0.01010847091674805</v>
+        <v>0.0008599758148193359</v>
       </c>
       <c r="U19" t="n">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="V19" t="n">
-        <v>0.0001430511474609375</v>
+        <v>1.668930053710938e-05</v>
       </c>
       <c r="W19" t="n">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="X19" t="n">
-        <v>0.0002002716064453125</v>
+        <v>2.121925354003906e-05</v>
       </c>
       <c r="Y19" t="n">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.0003759860992431641</v>
+        <v>0.0001132488250732422</v>
       </c>
       <c r="AA19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.002666473388671875</v>
+        <v>8.654594421386719e-05</v>
       </c>
       <c r="AC19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="AD19" t="n">
-        <v>0.002329349517822266</v>
+        <v>9.107589721679688e-05</v>
       </c>
       <c r="AE19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="AF19" t="n">
-        <v>0.0004189014434814453</v>
+        <v>5.316734313964844e-05</v>
       </c>
       <c r="AG19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="AH19" t="n">
-        <v>0.000453948974609375</v>
+        <v>4.315376281738281e-05</v>
       </c>
       <c r="AI19" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="AJ19" t="n">
-        <v>3.828750133514404</v>
+        <v>0.1733362674713135</v>
       </c>
       <c r="AK19" t="n">
         <v>0</v>
@@ -2770,110 +2770,110 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>N2W1B3R0.txt</t>
+          <t>N3W2B3R9.txt</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E20" t="n">
         <v>1000</v>
       </c>
       <c r="F20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0002381801605224609</v>
+        <v>0.0004837512969970703</v>
       </c>
       <c r="I20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0002102851867675781</v>
+        <v>0.00048828125</v>
       </c>
       <c r="K20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0002465248107910156</v>
+        <v>0.0004796981811523438</v>
       </c>
       <c r="M20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N20" t="n">
-        <v>0.0003390312194824219</v>
+        <v>0.0005791187286376953</v>
       </c>
       <c r="O20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="P20" t="n">
-        <v>0.0003399848937988281</v>
+        <v>0.0006823539733886719</v>
       </c>
       <c r="Q20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="R20" t="n">
-        <v>0.0004584789276123047</v>
+        <v>0.0007221698760986328</v>
       </c>
       <c r="S20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="T20" t="n">
-        <v>0.001760721206665039</v>
+        <v>0.00381159782409668</v>
       </c>
       <c r="U20" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="V20" t="n">
-        <v>3.695487976074219e-05</v>
+        <v>5.793571472167969e-05</v>
       </c>
       <c r="W20" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="X20" t="n">
-        <v>4.625320434570312e-05</v>
+        <v>9.012222290039062e-05</v>
       </c>
       <c r="Y20" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.0001585483551025391</v>
+        <v>0.0001924037933349609</v>
       </c>
       <c r="AA20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.0003085136413574219</v>
+        <v>0.0006787776947021484</v>
       </c>
       <c r="AC20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.0003151893615722656</v>
+        <v>0.0006875991821289062</v>
       </c>
       <c r="AE20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AF20" t="n">
-        <v>8.487701416015625e-05</v>
+        <v>0.0001626014709472656</v>
       </c>
       <c r="AG20" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AH20" t="n">
-        <v>9.441375732421875e-05</v>
+        <v>0.0001773834228515625</v>
       </c>
       <c r="AI20" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0.7133538722991943</v>
+        <v>1.226408243179321</v>
       </c>
       <c r="AK20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2889,110 +2889,110 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>N4W1B1R1.txt</t>
+          <t>N2W2B1R1.txt</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="E21" t="n">
         <v>1000</v>
       </c>
       <c r="F21" t="n">
-        <v>167</v>
+        <v>20</v>
       </c>
       <c r="G21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="H21" t="n">
-        <v>0.004356622695922852</v>
+        <v>0.00014495849609375</v>
       </c>
       <c r="I21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="J21" t="n">
-        <v>0.004128456115722656</v>
+        <v>0.0001330375671386719</v>
       </c>
       <c r="K21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="L21" t="n">
-        <v>0.002033233642578125</v>
+        <v>0.0001287460327148438</v>
       </c>
       <c r="M21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="N21" t="n">
-        <v>0.004104375839233398</v>
+        <v>0.0001876354217529297</v>
       </c>
       <c r="O21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="P21" t="n">
-        <v>0.006410360336303711</v>
+        <v>0.0001883506774902344</v>
       </c>
       <c r="Q21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="R21" t="n">
-        <v>0.005894660949707031</v>
+        <v>0.0002319812774658203</v>
       </c>
       <c r="S21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="T21" t="n">
-        <v>0.01194596290588379</v>
+        <v>0.002524137496948242</v>
       </c>
       <c r="U21" t="n">
-        <v>203</v>
+        <v>22</v>
       </c>
       <c r="V21" t="n">
-        <v>0.0001819133758544922</v>
+        <v>2.980232238769531e-05</v>
       </c>
       <c r="W21" t="n">
-        <v>203</v>
+        <v>22</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0002140998840332031</v>
+        <v>4.243850708007812e-05</v>
       </c>
       <c r="Y21" t="n">
-        <v>203</v>
+        <v>22</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.0004656314849853516</v>
+        <v>9.560585021972656e-05</v>
       </c>
       <c r="AA21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.005840301513671875</v>
+        <v>0.0001714229583740234</v>
       </c>
       <c r="AC21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.00566411018371582</v>
+        <v>0.0001804828643798828</v>
       </c>
       <c r="AE21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.0004558563232421875</v>
+        <v>7.724761962890625e-05</v>
       </c>
       <c r="AG21" t="n">
-        <v>184</v>
+        <v>22</v>
       </c>
       <c r="AH21" t="n">
-        <v>0.0004851818084716797</v>
+        <v>8.249282836914062e-05</v>
       </c>
       <c r="AI21" t="n">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="AJ21" t="n">
-        <v>10.05077314376831</v>
+        <v>0.3373570442199707</v>
       </c>
       <c r="AK21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3003,115 +3003,115 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Wäscher</t>
+          <t>Hard28</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Waescher_TEST0005.txt</t>
+          <t>Hard28_BPP359.txt</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>114</v>
+        <v>180</v>
       </c>
       <c r="E22" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F22" t="n">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="G22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0002069473266601562</v>
+        <v>0.000659942626953125</v>
       </c>
       <c r="I22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0001943111419677734</v>
+        <v>0.0006289482116699219</v>
       </c>
       <c r="K22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="L22" t="n">
-        <v>0.0001633167266845703</v>
+        <v>0.0007152557373046875</v>
       </c>
       <c r="M22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="N22" t="n">
-        <v>0.0009238719940185547</v>
+        <v>0.0008840560913085938</v>
       </c>
       <c r="O22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="P22" t="n">
-        <v>0.0003142356872558594</v>
+        <v>0.001199483871459961</v>
       </c>
       <c r="Q22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="R22" t="n">
-        <v>0.0003285408020019531</v>
+        <v>0.001228570938110352</v>
       </c>
       <c r="S22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="T22" t="n">
-        <v>0.01855874061584473</v>
+        <v>0.001958131790161133</v>
       </c>
       <c r="U22" t="n">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="V22" t="n">
-        <v>3.886222839355469e-05</v>
+        <v>5.578994750976562e-05</v>
       </c>
       <c r="W22" t="n">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="X22" t="n">
-        <v>5.841255187988281e-05</v>
+        <v>7.152557373046875e-05</v>
       </c>
       <c r="Y22" t="n">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.0007436275482177734</v>
+        <v>0.0003085136413574219</v>
       </c>
       <c r="AA22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.0003111362457275391</v>
+        <v>0.001173496246337891</v>
       </c>
       <c r="AC22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.0003108978271484375</v>
+        <v>0.001198530197143555</v>
       </c>
       <c r="AE22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="AF22" t="n">
-        <v>9.107589721679688e-05</v>
+        <v>0.0001394748687744141</v>
       </c>
       <c r="AG22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="AH22" t="n">
-        <v>9.822845458984375e-05</v>
+        <v>0.0001502037048339844</v>
       </c>
       <c r="AI22" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="AJ22" t="n">
-        <v>0.9665305614471436</v>
+        <v>1.859875679016113</v>
       </c>
       <c r="AK22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3122,115 +3122,115 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Hard28</t>
+          <t>Wäscher</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hard28_BPP60.txt</t>
+          <t>Waescher_TEST0055B.txt</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>160</v>
+        <v>239</v>
       </c>
       <c r="E23" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F23" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="G23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0006380081176757812</v>
+        <v>0.0003495216369628906</v>
       </c>
       <c r="I23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0005941390991210938</v>
+        <v>0.000362396240234375</v>
       </c>
       <c r="K23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="L23" t="n">
-        <v>0.0006439685821533203</v>
+        <v>0.0002381801605224609</v>
       </c>
       <c r="M23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0006606578826904297</v>
+        <v>0.0007932186126708984</v>
       </c>
       <c r="O23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0009126663208007812</v>
+        <v>0.0004944801330566406</v>
       </c>
       <c r="Q23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="R23" t="n">
-        <v>0.0009338855743408203</v>
+        <v>0.0005145072937011719</v>
       </c>
       <c r="S23" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="T23" t="n">
-        <v>0.007544755935668945</v>
+        <v>0.05354499816894531</v>
       </c>
       <c r="U23" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="V23" t="n">
-        <v>5.245208740234375e-05</v>
+        <v>7.081031799316406e-05</v>
       </c>
       <c r="W23" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="X23" t="n">
-        <v>7.033348083496094e-05</v>
+        <v>0.0001008510589599609</v>
       </c>
       <c r="Y23" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.0002069473266601562</v>
+        <v>0.0005180835723876953</v>
       </c>
       <c r="AA23" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="AB23" t="n">
-        <v>0.0008997917175292969</v>
+        <v>0.0006344318389892578</v>
       </c>
       <c r="AC23" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="AD23" t="n">
-        <v>0.00089263916015625</v>
+        <v>0.0005118846893310547</v>
       </c>
       <c r="AE23" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="AF23" t="n">
-        <v>0.0001270771026611328</v>
+        <v>0.0001864433288574219</v>
       </c>
       <c r="AG23" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="AH23" t="n">
-        <v>0.0001370906829833984</v>
+        <v>0.0002012252807617188</v>
       </c>
       <c r="AI23" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="AJ23" t="n">
-        <v>1.475684642791748</v>
+        <v>1.010661363601685</v>
       </c>
       <c r="AK23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -3241,112 +3241,112 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Wäscher</t>
+          <t>Hard28</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Waescher_TEST0014.txt</t>
+          <t>Hard28_BPP814.txt</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>96</v>
+        <v>200</v>
       </c>
       <c r="E24" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F24" t="n">
-        <v>23</v>
+        <v>81</v>
       </c>
       <c r="G24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0001685619354248047</v>
+        <v>0.0007433891296386719</v>
       </c>
       <c r="I24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0001456737518310547</v>
+        <v>0.0007174015045166016</v>
       </c>
       <c r="K24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0001332759857177734</v>
+        <v>0.0007979869842529297</v>
       </c>
       <c r="M24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="N24" t="n">
-        <v>0.001069784164428711</v>
+        <v>0.0008971691131591797</v>
       </c>
       <c r="O24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0002458095550537109</v>
+        <v>0.001443147659301758</v>
       </c>
       <c r="Q24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="R24" t="n">
-        <v>0.0002520084381103516</v>
+        <v>0.001527786254882812</v>
       </c>
       <c r="S24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="T24" t="n">
-        <v>0.01289868354797363</v>
+        <v>0.001933097839355469</v>
       </c>
       <c r="U24" t="n">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="V24" t="n">
-        <v>3.457069396972656e-05</v>
+        <v>6.008148193359375e-05</v>
       </c>
       <c r="W24" t="n">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="X24" t="n">
-        <v>0.0002415180206298828</v>
+        <v>8.58306884765625e-05</v>
       </c>
       <c r="Y24" t="n">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.004618406295776367</v>
+        <v>0.0002510547637939453</v>
       </c>
       <c r="AA24" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.0002925395965576172</v>
+        <v>0.00143742561340332</v>
       </c>
       <c r="AC24" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.0003049373626708984</v>
+        <v>0.001492738723754883</v>
       </c>
       <c r="AE24" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="AF24" t="n">
-        <v>9.5367431640625e-05</v>
+        <v>0.0001654624938964844</v>
       </c>
       <c r="AG24" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="AH24" t="n">
-        <v>0.0001006126403808594</v>
+        <v>0.0001728534698486328</v>
       </c>
       <c r="AI24" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="AJ24" t="n">
-        <v>0.5489509105682373</v>
+        <v>1.99487566947937</v>
       </c>
       <c r="AK24" t="n">
         <v>1</v>
@@ -3360,115 +3360,115 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hard28</t>
+          <t>Wäscher</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hard28_BPP144.txt</t>
+          <t>Waescher_TEST0097.txt</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>200</v>
+        <v>119</v>
       </c>
       <c r="E25" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F25" t="n">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="G25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0007901191711425781</v>
+        <v>0.0001189708709716797</v>
       </c>
       <c r="I25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0007817745208740234</v>
+        <v>0.0001196861267089844</v>
       </c>
       <c r="K25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="L25" t="n">
-        <v>0.0007941722869873047</v>
+        <v>0.0001132488250732422</v>
       </c>
       <c r="M25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0008640289306640625</v>
+        <v>0.0005617141723632812</v>
       </c>
       <c r="O25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="P25" t="n">
-        <v>0.001278877258300781</v>
+        <v>0.0002419948577880859</v>
       </c>
       <c r="Q25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="R25" t="n">
-        <v>0.001307249069213867</v>
+        <v>0.0002052783966064453</v>
       </c>
       <c r="S25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="T25" t="n">
-        <v>0.002939462661743164</v>
+        <v>0.02144169807434082</v>
       </c>
       <c r="U25" t="n">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="V25" t="n">
-        <v>6.031990051269531e-05</v>
+        <v>4.076957702636719e-05</v>
       </c>
       <c r="W25" t="n">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="X25" t="n">
-        <v>8.20159912109375e-05</v>
+        <v>5.555152893066406e-05</v>
       </c>
       <c r="Y25" t="n">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.0002346038818359375</v>
+        <v>0.0004301071166992188</v>
       </c>
       <c r="AA25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.001267910003662109</v>
+        <v>0.0001828670501708984</v>
       </c>
       <c r="AC25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="AD25" t="n">
-        <v>0.001511812210083008</v>
+        <v>0.0001940727233886719</v>
       </c>
       <c r="AE25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="AF25" t="n">
-        <v>0.0001778602600097656</v>
+        <v>8.988380432128906e-05</v>
       </c>
       <c r="AG25" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="AH25" t="n">
-        <v>0.0001802444458007812</v>
+        <v>9.870529174804688e-05</v>
       </c>
       <c r="AI25" t="n">
-        <v>75</v>
+        <v>13</v>
       </c>
       <c r="AJ25" t="n">
-        <v>2.004045486450195</v>
+        <v>0.3084621429443359</v>
       </c>
       <c r="AK25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -3479,112 +3479,112 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Hard28</t>
+          <t>Wäscher</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hard28_BPP195.txt</t>
+          <t>Waescher_TEST0014.txt</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>180</v>
+        <v>96</v>
       </c>
       <c r="E26" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F26" t="n">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="G26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0006196498870849609</v>
+        <v>0.0001492500305175781</v>
       </c>
       <c r="I26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0005757808685302734</v>
+        <v>0.0001397132873535156</v>
       </c>
       <c r="K26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="L26" t="n">
-        <v>0.0008463859558105469</v>
+        <v>0.0001327991485595703</v>
       </c>
       <c r="M26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="N26" t="n">
-        <v>0.0007464885711669922</v>
+        <v>0.0008549690246582031</v>
       </c>
       <c r="O26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="P26" t="n">
-        <v>0.001129865646362305</v>
+        <v>0.0002431869506835938</v>
       </c>
       <c r="Q26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="R26" t="n">
-        <v>0.001140117645263672</v>
+        <v>0.0002732276916503906</v>
       </c>
       <c r="S26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="T26" t="n">
-        <v>0.002351522445678711</v>
+        <v>0.01792144775390625</v>
       </c>
       <c r="U26" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="V26" t="n">
-        <v>5.483627319335938e-05</v>
+        <v>3.910064697265625e-05</v>
       </c>
       <c r="W26" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="X26" t="n">
-        <v>7.367134094238281e-05</v>
+        <v>4.458427429199219e-05</v>
       </c>
       <c r="Y26" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.0003392696380615234</v>
+        <v>0.0007166862487792969</v>
       </c>
       <c r="AA26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.001153469085693359</v>
+        <v>0.0002255439758300781</v>
       </c>
       <c r="AC26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.001168489456176758</v>
+        <v>0.0002439022064208984</v>
       </c>
       <c r="AE26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="AF26" t="n">
-        <v>0.0001485347747802734</v>
+        <v>8.0108642578125e-05</v>
       </c>
       <c r="AG26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="AH26" t="n">
-        <v>0.0001599788665771484</v>
+        <v>8.177757263183594e-05</v>
       </c>
       <c r="AI26" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="AJ26" t="n">
-        <v>1.634788990020752</v>
+        <v>0.3803062438964844</v>
       </c>
       <c r="AK26" t="n">
         <v>1</v>
@@ -3598,115 +3598,115 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>set_3</t>
+          <t>Hard28</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HARD5.txt</t>
+          <t>Hard28_BPP645.txt</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="E27" t="n">
-        <v>100000</v>
+        <v>1000</v>
       </c>
       <c r="F27" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G27" t="n">
         <v>59</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0006198883056640625</v>
+        <v>0.0005054473876953125</v>
       </c>
       <c r="I27" t="n">
         <v>59</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0007474422454833984</v>
+        <v>0.0004830360412597656</v>
       </c>
       <c r="K27" t="n">
         <v>59</v>
       </c>
       <c r="L27" t="n">
-        <v>0.0007102489471435547</v>
+        <v>0.0005030632019042969</v>
       </c>
       <c r="M27" t="n">
         <v>59</v>
       </c>
       <c r="N27" t="n">
-        <v>0.1427755355834961</v>
+        <v>0.0006852149963378906</v>
       </c>
       <c r="O27" t="n">
         <v>59</v>
       </c>
       <c r="P27" t="n">
-        <v>0.0008308887481689453</v>
+        <v>0.0008378028869628906</v>
       </c>
       <c r="Q27" t="n">
         <v>59</v>
       </c>
       <c r="R27" t="n">
-        <v>0.0008187294006347656</v>
+        <v>0.0008552074432373047</v>
       </c>
       <c r="S27" t="n">
         <v>59</v>
       </c>
       <c r="T27" t="n">
-        <v>0.5676488876342773</v>
+        <v>0.002398967742919922</v>
       </c>
       <c r="U27" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="V27" t="n">
-        <v>7.534027099609375e-05</v>
+        <v>4.9591064453125e-05</v>
       </c>
       <c r="W27" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="X27" t="n">
-        <v>8.893013000488281e-05</v>
+        <v>6.437301635742188e-05</v>
       </c>
       <c r="Y27" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.005671262741088867</v>
+        <v>0.0002655982971191406</v>
       </c>
       <c r="AA27" t="n">
         <v>59</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.0008056163787841797</v>
+        <v>0.0008268356323242188</v>
       </c>
       <c r="AC27" t="n">
         <v>59</v>
       </c>
       <c r="AD27" t="n">
-        <v>0.0008256435394287109</v>
+        <v>0.0008540153503417969</v>
       </c>
       <c r="AE27" t="n">
         <v>59</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.0001630783081054688</v>
+        <v>0.0001280307769775391</v>
       </c>
       <c r="AG27" t="n">
         <v>59</v>
       </c>
       <c r="AH27" t="n">
-        <v>0.0001776218414306641</v>
+        <v>0.0001344680786132812</v>
       </c>
       <c r="AI27" t="n">
         <v>59</v>
       </c>
       <c r="AJ27" t="n">
-        <v>1.717100620269775</v>
+        <v>1.3453209400177</v>
       </c>
       <c r="AK27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3717,115 +3717,115 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>set_3</t>
+          <t>Wäscher</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HARD3.txt</t>
+          <t>Waescher_TEST0022.txt</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>200</v>
+        <v>57</v>
       </c>
       <c r="E28" t="n">
-        <v>100000</v>
+        <v>10000</v>
       </c>
       <c r="F28" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="G28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0006923675537109375</v>
+        <v>8.082389831542969e-05</v>
       </c>
       <c r="I28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0007064342498779297</v>
+        <v>6.055831909179688e-05</v>
       </c>
       <c r="K28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="L28" t="n">
-        <v>0.0009148120880126953</v>
+        <v>7.05718994140625e-05</v>
       </c>
       <c r="M28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="N28" t="n">
-        <v>0.2405679225921631</v>
+        <v>0.0007538795471191406</v>
       </c>
       <c r="O28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="P28" t="n">
-        <v>0.001105308532714844</v>
+        <v>0.0001146793365478516</v>
       </c>
       <c r="Q28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="R28" t="n">
-        <v>0.001042366027832031</v>
+        <v>0.0001015663146972656</v>
       </c>
       <c r="S28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="T28" t="n">
-        <v>0.9407944679260254</v>
+        <v>0.009706974029541016</v>
       </c>
       <c r="U28" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="V28" t="n">
-        <v>8.0108642578125e-05</v>
+        <v>2.050399780273438e-05</v>
       </c>
       <c r="W28" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="X28" t="n">
-        <v>9.5367431640625e-05</v>
+        <v>2.956390380859375e-05</v>
       </c>
       <c r="Y28" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.01189112663269043</v>
+        <v>0.0006711483001708984</v>
       </c>
       <c r="AA28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.0008947849273681641</v>
+        <v>0.0001058578491210938</v>
       </c>
       <c r="AC28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="AD28" t="n">
-        <v>0.00107264518737793</v>
+        <v>9.846687316894531e-05</v>
       </c>
       <c r="AE28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="AF28" t="n">
-        <v>0.0002360343933105469</v>
+        <v>4.601478576660156e-05</v>
       </c>
       <c r="AG28" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="AH28" t="n">
-        <v>0.0002648830413818359</v>
+        <v>4.553794860839844e-05</v>
       </c>
       <c r="AI28" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="AJ28" t="n">
-        <v>1.883800506591797</v>
+        <v>0.1564033031463623</v>
       </c>
       <c r="AK28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3836,112 +3836,112 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Wäscher</t>
+          <t>Hard28</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Waescher_TEST0082.txt</t>
+          <t>Hard28_BPP47.txt</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>86</v>
+        <v>180</v>
       </c>
       <c r="E29" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F29" t="n">
-        <v>24</v>
+        <v>71</v>
       </c>
       <c r="G29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0001485347747802734</v>
+        <v>0.0007231235504150391</v>
       </c>
       <c r="I29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0001366138458251953</v>
+        <v>0.0005774497985839844</v>
       </c>
       <c r="K29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="L29" t="n">
-        <v>0.0001263618469238281</v>
+        <v>0.0006535053253173828</v>
       </c>
       <c r="M29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="N29" t="n">
-        <v>0.001140117645263672</v>
+        <v>0.0007600784301757812</v>
       </c>
       <c r="O29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="P29" t="n">
-        <v>0.0002329349517822266</v>
+        <v>0.001227617263793945</v>
       </c>
       <c r="Q29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="R29" t="n">
-        <v>0.0002398490905761719</v>
+        <v>0.0011749267578125</v>
       </c>
       <c r="S29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="T29" t="n">
-        <v>0.01479649543762207</v>
+        <v>0.002092361450195312</v>
       </c>
       <c r="U29" t="n">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="V29" t="n">
-        <v>3.123283386230469e-05</v>
+        <v>5.817413330078125e-05</v>
       </c>
       <c r="W29" t="n">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="X29" t="n">
-        <v>4.339218139648438e-05</v>
+        <v>7.796287536621094e-05</v>
       </c>
       <c r="Y29" t="n">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.0009944438934326172</v>
+        <v>0.0002300739288330078</v>
       </c>
       <c r="AA29" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.0002236366271972656</v>
+        <v>0.001152515411376953</v>
       </c>
       <c r="AC29" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="AD29" t="n">
-        <v>0.0002396106719970703</v>
+        <v>0.001215219497680664</v>
       </c>
       <c r="AE29" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="AF29" t="n">
-        <v>7.009506225585938e-05</v>
+        <v>0.0001478195190429688</v>
       </c>
       <c r="AG29" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="AH29" t="n">
-        <v>7.295608520507812e-05</v>
+        <v>0.0001578330993652344</v>
       </c>
       <c r="AI29" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0.6750619411468506</v>
+        <v>1.676855087280273</v>
       </c>
       <c r="AK29" t="n">
         <v>1</v>
@@ -3955,112 +3955,112 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Wäscher</t>
+          <t>set_3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Waescher_TEST0084.txt</t>
+          <t>HARD8.txt</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>92</v>
+        <v>200</v>
       </c>
       <c r="E30" t="n">
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="F30" t="n">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="G30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="H30" t="n">
-        <v>0.00012969970703125</v>
+        <v>0.0005893707275390625</v>
       </c>
       <c r="I30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0001206398010253906</v>
+        <v>0.0005807876586914062</v>
       </c>
       <c r="K30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0001287460327148438</v>
+        <v>0.0006916522979736328</v>
       </c>
       <c r="M30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="N30" t="n">
-        <v>0.002035856246948242</v>
+        <v>0.006161689758300781</v>
       </c>
       <c r="O30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="P30" t="n">
-        <v>0.0001742839813232422</v>
+        <v>0.0007967948913574219</v>
       </c>
       <c r="Q30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="R30" t="n">
-        <v>0.00018310546875</v>
+        <v>0.0008068084716796875</v>
       </c>
       <c r="S30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="T30" t="n">
-        <v>0.02448773384094238</v>
+        <v>0.4185693264007568</v>
       </c>
       <c r="U30" t="n">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="V30" t="n">
-        <v>8.749961853027344e-05</v>
+        <v>7.724761962890625e-05</v>
       </c>
       <c r="W30" t="n">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="X30" t="n">
-        <v>5.674362182617188e-05</v>
+        <v>9.036064147949219e-05</v>
       </c>
       <c r="Y30" t="n">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.007002115249633789</v>
+        <v>0.1252350807189941</v>
       </c>
       <c r="AA30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.0001966953277587891</v>
+        <v>0.0007987022399902344</v>
       </c>
       <c r="AC30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="AD30" t="n">
-        <v>0.0003342628479003906</v>
+        <v>0.0008325576782226562</v>
       </c>
       <c r="AE30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="AF30" t="n">
-        <v>8.869171142578125e-05</v>
+        <v>0.0001666545867919922</v>
       </c>
       <c r="AG30" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="AH30" t="n">
-        <v>9.679794311523438e-05</v>
+        <v>0.0001816749572753906</v>
       </c>
       <c r="AI30" t="n">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.3090920448303223</v>
+        <v>1.539526700973511</v>
       </c>
       <c r="AK30" t="n">
         <v>1</v>
@@ -4074,112 +4074,112 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Wäscher</t>
+          <t>Hard28</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Waescher_TEST0055A.txt</t>
+          <t>Hard28_BPP485.txt</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="E31" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F31" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="G31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0002086162567138672</v>
+        <v>0.0008168220520019531</v>
       </c>
       <c r="I31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0002031326293945312</v>
+        <v>0.0006766319274902344</v>
       </c>
       <c r="K31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="L31" t="n">
-        <v>0.0001738071441650391</v>
+        <v>0.0007450580596923828</v>
       </c>
       <c r="M31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="N31" t="n">
-        <v>0.0007150173187255859</v>
+        <v>0.00103306770324707</v>
       </c>
       <c r="O31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="P31" t="n">
-        <v>0.0002930164337158203</v>
+        <v>0.001202821731567383</v>
       </c>
       <c r="Q31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="R31" t="n">
-        <v>0.0003116130828857422</v>
+        <v>0.001562833786010742</v>
       </c>
       <c r="S31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="T31" t="n">
-        <v>0.03208446502685547</v>
+        <v>0.00255584716796875</v>
       </c>
       <c r="U31" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="V31" t="n">
-        <v>5.435943603515625e-05</v>
+        <v>8.106231689453125e-05</v>
       </c>
       <c r="W31" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="X31" t="n">
-        <v>7.724761962890625e-05</v>
+        <v>0.0001051425933837891</v>
       </c>
       <c r="Y31" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.0005614757537841797</v>
+        <v>0.0003595352172851562</v>
       </c>
       <c r="AA31" t="n">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.0003428459167480469</v>
+        <v>0.001489877700805664</v>
       </c>
       <c r="AC31" t="n">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="AD31" t="n">
-        <v>0.0003178119659423828</v>
+        <v>0.001498937606811523</v>
       </c>
       <c r="AE31" t="n">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="AF31" t="n">
-        <v>0.0001325607299804688</v>
+        <v>0.0002231597900390625</v>
       </c>
       <c r="AG31" t="n">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="AH31" t="n">
-        <v>0.0001494884490966797</v>
+        <v>0.0002624988555908203</v>
       </c>
       <c r="AI31" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="AJ31" t="n">
-        <v>0.5864715576171875</v>
+        <v>1.744535684585571</v>
       </c>
       <c r="AK31" t="n">
         <v>1</v>

</xml_diff>